<commit_message>
Deep remove old 2020 material upload A4 2022
</commit_message>
<xml_diff>
--- a/training schedule_cv_part_not_updated.xlsx
+++ b/training schedule_cv_part_not_updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guyle\Documents\Projects\CV_training\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18E02F95-4F58-477B-9B9C-06154483A278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7010512E-32B1-4432-8A54-EA6EA76E158E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1125" yWindow="1125" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -275,7 +275,7 @@
     <t>10.6-16.6</t>
   </si>
   <si>
-    <t>17.6-?</t>
+    <t>17.6-20.6</t>
   </si>
 </sst>
 </file>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="C32" s="16">
         <f>SUM(C33,C40,C44)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D32" s="16"/>
     </row>
@@ -1635,7 +1635,7 @@
       </c>
       <c r="C33" s="6">
         <f>SUM(C34:C39)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D33" s="6"/>
     </row>
@@ -1684,12 +1684,23 @@
       <c r="B36" s="4">
         <v>3</v>
       </c>
-      <c r="C36" s="4"/>
+      <c r="C36" s="4">
+        <v>2</v>
+      </c>
       <c r="D36" s="4" t="s">
         <v>22</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>79</v>
+      </c>
+      <c r="F36" s="2">
+        <v>4</v>
+      </c>
+      <c r="G36" s="2">
+        <v>5</v>
+      </c>
+      <c r="H36" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>